<commit_message>
Improve public prayer experience
</commit_message>
<xml_diff>
--- a/output/spreadsheet/startpray-progress-tracker.xlsx
+++ b/output/spreadsheet/startpray-progress-tracker.xlsx
@@ -599,7 +599,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>dee4b64</t>
+          <t>fd5493d</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10 19:36:25</t>
+          <t>2026-05-23 12:03:24</t>
         </is>
       </c>
     </row>
@@ -3647,7 +3647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4267,14 +4267,80 @@
           <t>[AUTO] Commit recorded: main @ dee4b64</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
           <t>Continue task updates and prepare push.</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-05-12 23:39:45</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: main @ b6d027d</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-05-23 12:03:01</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: main @ ae2e854</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-05-23 12:03:24</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: main @ fd5493d</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
         <is>
           <t>git-hook</t>
         </is>
@@ -4411,7 +4477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5432,7 +5498,118 @@
           <t>https://github.com/dan40912/Start-Pray.git</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-05-12 23:39:45</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>b6d027d</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Improve prayer sharing reports and guest posting</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/Start-Pray.git</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-05-23 12:03:01</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>ae2e854</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Improve public prayer experience</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/Start-Pray.git</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-05-23 12:03:24</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>fd5493d</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Improve public prayer experience</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/Start-Pray.git</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Release Start Pray 2.1.0
Bump package version from 2.0.0 to 2.1.0.

Stabilize the homepage globe by replacing the duplicate fake earth overlay with a dedicated loading treatment, hiding Cesium canvas until ready, loading real map tiles under the loading artwork, and using a lighter hero-map mode with fewer markers and reduced per-frame work.

Improve guest prayer creation by making the submit action show a clear terms-required prompt and focus the acknowledgement checkbox before submission.

Update the Traditional Chinese homepage hero copy and refresh the progress tracker spreadsheet.
</commit_message>
<xml_diff>
--- a/output/spreadsheet/startpray-progress-tracker.xlsx
+++ b/output/spreadsheet/startpray-progress-tracker.xlsx
@@ -599,7 +599,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>fd5493d</t>
+          <t>2899667</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-23 12:03:24</t>
+          <t>2026-05-30 18:44:48</t>
         </is>
       </c>
     </row>
@@ -3647,7 +3647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4333,14 +4333,124 @@
           <t>[AUTO] Commit recorded: main @ fd5493d</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
           <t>Continue task updates and prepare push.</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-05-30 09:13:43</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: main @ 9d44c72</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-05-30 09:39:39</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: main @ 7aef01f</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-05-30 09:42:51</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: main @ a27271e</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-05-30 18:44:11</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: main @ aa29e0b</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-05-30 18:44:48</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: main @ 2899667</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
         <is>
           <t>git-hook</t>
         </is>
@@ -4477,7 +4587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5609,7 +5719,192 @@
           <t>https://github.com/dan40912/Start-Pray.git</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-05-30 09:13:43</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>9d44c72</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Improve localized prayer room experience</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/Start-Pray.git</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-05-30 09:39:39</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>7aef01f</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Stabilize homepage globe and prod deploy</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/Start-Pray.git</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-05-30 09:42:51</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>a27271e</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Start global prayer room from Taiwan</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/Start-Pray.git</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-05-30 18:44:11</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>aa29e0b</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Release Start Pray 2.1.0</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/Start-Pray.git</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-05-30 18:44:48</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>2899667</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Release Start Pray 2.1.0</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/Start-Pray.git</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Stabilize global prayer room map loading
Hide the Cesium canvas until the globe is ready and make the loading skeleton background opaque enough to prevent tile-loading redraws from flashing through.
</commit_message>
<xml_diff>
--- a/output/spreadsheet/startpray-progress-tracker.xlsx
+++ b/output/spreadsheet/startpray-progress-tracker.xlsx
@@ -599,7 +599,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>2899667</t>
+          <t>457fe5d</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-30 18:44:48</t>
+          <t>2026-05-30 18:57:53</t>
         </is>
       </c>
     </row>
@@ -3647,7 +3647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4443,14 +4443,36 @@
           <t>[AUTO] Commit recorded: main @ 2899667</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
           <t>Continue task updates and prepare push.</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-05-30 18:57:53</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: main @ 457fe5d</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
         <is>
           <t>git-hook</t>
         </is>
@@ -4587,7 +4609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5904,7 +5926,44 @@
           <t>https://github.com/dan40912/Start-Pray.git</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-05-30 18:57:53</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>457fe5d</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Stabilize global prayer room map loading</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/Start-Pray.git</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update project progress tracker
</commit_message>
<xml_diff>
--- a/output/spreadsheet/startpray-progress-tracker.xlsx
+++ b/output/spreadsheet/startpray-progress-tracker.xlsx
@@ -582,7 +582,7 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>feature/roadmap-prd-implementation</t>
         </is>
       </c>
     </row>
@@ -599,7 +599,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>457fe5d</t>
+          <t>753a726</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-30 18:57:53</t>
+          <t>2026-07-14 23:16:44</t>
         </is>
       </c>
     </row>
@@ -3647,7 +3647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4465,14 +4465,36 @@
           <t>[AUTO] Commit recorded: main @ 457fe5d</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
           <t>Continue task updates and prepare push.</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-07-14 23:16:44</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: feature/roadmap-prd-implementation @ 753a726</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
         <is>
           <t>git-hook</t>
         </is>
@@ -4609,7 +4631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5963,7 +5985,44 @@
           <t>https://github.com/dan40912/Start-Pray.git</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-07-14 23:16:44</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>feature/roadmap-prd-implementation</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>753a726</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Implement roadmap PRDs and prayer experience updates</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/Start-Pray.git</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update project progress tracker after merge
</commit_message>
<xml_diff>
--- a/output/spreadsheet/startpray-progress-tracker.xlsx
+++ b/output/spreadsheet/startpray-progress-tracker.xlsx
@@ -582,7 +582,7 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>feature/roadmap-prd-implementation</t>
+          <t>main</t>
         </is>
       </c>
     </row>
@@ -599,7 +599,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>8068c33</t>
+          <t>89bcc02</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>2026-07-14 23:45:50</t>
+          <t>2026-07-15 00:07:16</t>
         </is>
       </c>
     </row>
@@ -3647,7 +3647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4509,14 +4509,36 @@
           <t>[AUTO] Commit recorded: feature/roadmap-prd-implementation @ 8068c33</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
           <t>Continue task updates and prepare push.</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-07-15 00:07:16</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: main @ 89bcc02</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
         <is>
           <t>git-hook</t>
         </is>
@@ -4653,7 +4675,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6081,7 +6103,44 @@
           <t>https://github.com/dan40912/Start-Pray.git</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-07-15 00:07:16</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>89bcc02</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Merge feature/roadmap-prd-implementation into main</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/Start-Pray.git</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs: record what phase 0 landed and hand the rest to the three tracks
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/spreadsheet/startpray-progress-tracker.xlsx
+++ b/output/spreadsheet/startpray-progress-tracker.xlsx
@@ -599,7 +599,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>32a60d6</t>
+          <t>6364fd9</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>2026-09-10 01:03:36</t>
+          <t>2026-09-10 01:08:25</t>
         </is>
       </c>
     </row>
@@ -3647,7 +3647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F64"/>
+  <dimension ref="A1:F65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5059,14 +5059,36 @@
           <t>[AUTO] Commit recorded: design/phase0-foundation @ 32a60d6</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr"/>
-      <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr">
         <is>
           <t>Continue task updates and prepare push.</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-09-10 01:08:25</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: design/phase0-foundation @ 6364fd9</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
         <is>
           <t>git-hook</t>
         </is>
@@ -5203,7 +5225,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H63"/>
+  <dimension ref="A1:H64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7556,7 +7578,44 @@
           <t>https://github.com/dan40912/Start-Pray.git</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-09-10 01:08:25</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>design/phase0-foundation</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>6364fd9</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>refactor(design): share one card component, keep one CTA per screen</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/Start-Pray.git</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix(prayer-room): stop the map controls stretching across the globe
`.gpr-page__map-controls` is a wrapping flex row, and flex defaults
`align-items` and `align-content` to stretch, so once the six buttons wrapped
onto three lines each one grew to 211px tall and the stack covered the globe.
The container was also 647px of transparent overlay sitting in front of the
map, which would have eaten drags meant for the globe itself.

Also records the finished work in DESIGN_COORDINATION.md, including the two
things I did not do: the signed-in portal screens are unverified in a browser,
and the seed-response volume is untouched.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/spreadsheet/startpray-progress-tracker.xlsx
+++ b/output/spreadsheet/startpray-progress-tracker.xlsx
@@ -599,7 +599,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>a22d0ff</t>
+          <t>372571e</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>2026-09-10 01:39:55</t>
+          <t>2026-09-10 01:41:49</t>
         </is>
       </c>
     </row>
@@ -3647,7 +3647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F70"/>
+  <dimension ref="A1:F71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5191,14 +5191,36 @@
           <t>[AUTO] Commit recorded: design/phase0-foundation @ a22d0ff</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr"/>
-      <c r="D70" t="inlineStr"/>
       <c r="E70" t="inlineStr">
         <is>
           <t>Continue task updates and prepare push.</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-09-10 01:41:49</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: design/phase0-foundation @ 372571e</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
         <is>
           <t>git-hook</t>
         </is>
@@ -5335,7 +5357,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H69"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7910,7 +7932,44 @@
           <t>https://github.com/dan40912/Start-Pray.git</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-09-10 01:41:49</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>design/phase0-foundation</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>372571e</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>refactor(routes): the member area is /me, not /customer-portal</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/Start-Pray.git</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(prayer): hide the "我已為你禱告" reaction
Pressing it changes nothing anyone can feel — not for the person who wrote the
prayer, not for the person pressing it — so it was one more control to work out
on a screen that should ask for exactly one thing. It goes from the home hero
and the detail panel, taking its count line with it.

Nothing is deleted: `PrayedReactionButton`, `usePrayedReaction` and
`/api/home-cards/:id/prayed` all stay, along with every reaction already
recorded. Putting the line back turns it on again.

The anonymity note underneath ("匿名送出，你可以在送出前重新錄製。") is kept —
it explains how sending works rather than belonging to the button.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/spreadsheet/startpray-progress-tracker.xlsx
+++ b/output/spreadsheet/startpray-progress-tracker.xlsx
@@ -599,7 +599,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>372571e</t>
+          <t>869055a</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>2026-09-10 01:41:49</t>
+          <t>2026-09-10 01:45:30</t>
         </is>
       </c>
     </row>
@@ -3647,7 +3647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:F72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5213,14 +5213,36 @@
           <t>[AUTO] Commit recorded: design/phase0-foundation @ 372571e</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr"/>
-      <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr">
         <is>
           <t>Continue task updates and prepare push.</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-09-10 01:45:30</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: design/phase0-foundation @ 869055a</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
         <is>
           <t>git-hook</t>
         </is>
@@ -5357,7 +5379,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H70"/>
+  <dimension ref="A1:H71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7969,7 +7991,44 @@
           <t>https://github.com/dan40912/Start-Pray.git</t>
         </is>
       </c>
-      <c r="H70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-09-10 01:45:30</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>design/phase0-foundation</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>869055a</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>fix(prayer-room): stop the map controls stretching across the globe</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/Start-Pray.git</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>